<commit_message>
MAJ avec les plafonds 2026 pour revenus 2025
</commit_message>
<xml_diff>
--- a/Simulateur Impôt 2025.xlsx
+++ b/Simulateur Impôt 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://15041946-my.sharepoint.com/personal/guillaume_guilbert_ext_plasticomnium_com/Documents/Documents/000-Perso/Conseil patrimoine/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://15041946-my.sharepoint.com/personal/guillaume_guilbert_ext_plasticomnium_com/Documents/Documents/000-Perso/Conseil patrimoine/Outils/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{C0528B22-4170-4882-BFF7-495ED349E4EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD9327CE-AB7F-4CA6-BE02-A86B68AB9EA8}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{C0528B22-4170-4882-BFF7-495ED349E4EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F2F2342-32C9-48AC-BB47-1C35A3B24D74}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{F929243B-59AF-4C27-884B-2E1D5A5CA125}"/>
+    <workbookView minimized="1" xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="9960" activeTab="2" xr2:uid="{F929243B-59AF-4C27-884B-2E1D5A5CA125}"/>
   </bookViews>
   <sheets>
     <sheet name="MAJ" sheetId="3" r:id="rId1"/>
@@ -333,7 +333,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="128">
   <si>
     <t>Situation de famille</t>
   </si>
@@ -789,6 +789,9 @@
   </si>
   <si>
     <t>Versement FCPI</t>
+  </si>
+  <si>
+    <t>Pinel</t>
   </si>
 </sst>
 </file>
@@ -2140,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="4">
-        <v>11497</v>
+        <v>11600</v>
       </c>
       <c r="C3" s="18">
         <v>0</v>
@@ -2157,10 +2160,11 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="17">
-        <v>11497</v>
+        <f>B3</f>
+        <v>11600</v>
       </c>
       <c r="B4" s="4">
-        <v>29315</v>
+        <v>29579</v>
       </c>
       <c r="C4" s="18">
         <v>0.11</v>
@@ -2177,10 +2181,11 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="17">
-        <v>29315</v>
+        <f>B4</f>
+        <v>29579</v>
       </c>
       <c r="B5" s="4">
-        <v>83823</v>
+        <v>54577</v>
       </c>
       <c r="C5" s="18">
         <v>0.3</v>
@@ -2192,10 +2197,11 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="17">
-        <v>83823</v>
+        <f>B5</f>
+        <v>54577</v>
       </c>
       <c r="B6" s="4">
-        <v>180294</v>
+        <v>181917</v>
       </c>
       <c r="C6" s="18">
         <v>0.41</v>
@@ -2207,7 +2213,8 @@
     </row>
     <row r="7" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19">
-        <v>180294</v>
+        <f>B6</f>
+        <v>181917</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21">
@@ -2282,7 +2289,7 @@
         <v>21</v>
       </c>
       <c r="B17" s="31">
-        <v>1791</v>
+        <v>1807</v>
       </c>
       <c r="D17" s="28" t="s">
         <v>39</v>
@@ -2295,7 +2302,8 @@
         <v>36</v>
       </c>
       <c r="B18" s="32">
-        <v>3582</v>
+        <f>B17*2</f>
+        <v>3614</v>
       </c>
       <c r="D18" s="29" t="s">
         <v>40</v>
@@ -2679,7 +2687,7 @@
     <col min="6" max="6" width="7.44140625" customWidth="1"/>
     <col min="7" max="7" width="51.6640625" customWidth="1"/>
     <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
@@ -2906,7 +2914,7 @@
         <v>121</v>
       </c>
       <c r="K13" s="93">
-        <f>IF(IF($H$11&gt;Données!B3,Données!B3,$H$11-Données!A3)&lt;0,0,IF($H$11&gt;Données!B3,Données!B3,$H$11-Données!A3))</f>
+        <f>IF(IF($H$11/C30&gt;Données!B3,Données!B3,Données!A3)&lt;0,0,IF($H$11/C30&gt;Données!B3,Données!B3,$H$11/C30-Données!A3))</f>
         <v>0</v>
       </c>
     </row>
@@ -2934,7 +2942,7 @@
         <v>122</v>
       </c>
       <c r="K14" s="93">
-        <f>IF(IF($H$11&gt;Données!B4,Données!B4,$H$11-Données!A4)&lt;0,0,IF($H$11&gt;Données!B4,Données!B4,$H$11-Données!A4))</f>
+        <f>IF(IF($H$11/C30&gt;Données!B4,Données!B4,$H$11/C30-Données!A4)&lt;0,0,IF($H$11/C30&gt;Données!B4,Données!B4,$H$11/C30-Données!A4))</f>
         <v>0</v>
       </c>
     </row>
@@ -2963,7 +2971,7 @@
         <v>123</v>
       </c>
       <c r="K15" s="93">
-        <f>IF(IF($H$11&gt;Données!B5,Données!B5,$H$11-Données!A5)&lt;0,0,IF($H$11&gt;Données!B5,Données!B5,$H$11-Données!A5))</f>
+        <f>IF(IF($H$11/C30&gt;Données!B5,Données!B5,$H$11/C30-Données!A5)&lt;0,0,IF($H$11/C30&gt;Données!B5,Données!B5,$H$11/C30-Données!A5))</f>
         <v>0</v>
       </c>
     </row>
@@ -2982,7 +2990,7 @@
         <v>124</v>
       </c>
       <c r="K16" s="93">
-        <f>IF(IF($H$11&gt;Données!B6,Données!B6,$H$11-Données!A6)&lt;0,0,IF($H$11&gt;Données!B6,Données!B6,$H$11-Données!A6))</f>
+        <f>IF(IF($H$11/C30&gt;Données!B6,Données!B6,$H$11/C30-Données!A6)&lt;0,0,IF($H$11/C30&gt;Données!B6,Données!B6,$H$11/C30-Données!A6))</f>
         <v>0</v>
       </c>
     </row>
@@ -3006,7 +3014,7 @@
         <v>125</v>
       </c>
       <c r="K17" s="93">
-        <f>IF((H11-Données!A7)&lt;0,0,H11-Données!A7)</f>
+        <f>IF((H11/C30-Données!A7)&lt;0,0,H11/C30-Données!A7)</f>
         <v>0</v>
       </c>
     </row>
@@ -3024,6 +3032,9 @@
       <c r="I18" t="s">
         <v>126</v>
       </c>
+      <c r="J18" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="106"/>
@@ -3042,10 +3053,13 @@
         <v>30</v>
       </c>
       <c r="H19" s="58">
-        <f>0.225*I19</f>
+        <f>0.225*I19+J19</f>
         <v>0</v>
       </c>
       <c r="I19" s="94">
+        <v>0</v>
+      </c>
+      <c r="J19" s="94">
         <v>0</v>
       </c>
     </row>
@@ -3220,7 +3234,7 @@
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="5">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{61FF6B5B-76F5-47A6-B377-712765BBC03B}">
           <x14:formula1>
             <xm:f>Données!$A$10:$A$14</xm:f>
@@ -3310,7 +3324,7 @@
       </c>
       <c r="F4" s="79">
         <f>MAX(B17:B18)</f>
-        <v>2079.9900000000002</v>
+        <v>2046</v>
       </c>
       <c r="I4" s="34" t="s">
         <v>115</v>
@@ -3344,7 +3358,7 @@
       </c>
       <c r="J5" s="4">
         <f>Données!B3</f>
-        <v>11497</v>
+        <v>11600</v>
       </c>
       <c r="K5" s="18">
         <v>0</v>
@@ -3369,11 +3383,11 @@
       </c>
       <c r="I6" s="17">
         <f>Données!A4</f>
-        <v>11497</v>
+        <v>11600</v>
       </c>
       <c r="J6" s="4">
         <f>Données!B4</f>
-        <v>29315</v>
+        <v>29579</v>
       </c>
       <c r="K6" s="18">
         <v>0.11</v>
@@ -3389,11 +3403,11 @@
       <c r="C7" s="1"/>
       <c r="I7" s="17">
         <f>Données!A5</f>
-        <v>29315</v>
+        <v>29579</v>
       </c>
       <c r="J7" s="4">
         <f>Données!B5</f>
-        <v>83823</v>
+        <v>54577</v>
       </c>
       <c r="K7" s="18">
         <v>0.3</v>
@@ -3405,16 +3419,16 @@
       </c>
       <c r="E8" s="83">
         <f>IF(AND(OR(B4='Simulateur impôt simplifié 2025'!I13,B4='Simulateur impôt simplifié 2025'!I16,B4='Simulateur impôt simplifié 2025'!I17),F4&lt;='Simulateur impôt simplifié 2025'!J31),F16,IF(AND(OR(B4='Simulateur impôt simplifié 2025'!I14,B4='Simulateur impôt simplifié 2025'!I15),F4&lt;='Simulateur impôt simplifié 2025'!J32),F17,0))</f>
-        <v>528.8045249999999</v>
+        <v>544.18499999999995</v>
       </c>
       <c r="F8" s="9"/>
       <c r="I8" s="17">
         <f>Données!A6</f>
-        <v>83823</v>
+        <v>54577</v>
       </c>
       <c r="J8" s="4">
         <f>Données!B6</f>
-        <v>180294</v>
+        <v>181917</v>
       </c>
       <c r="K8" s="18">
         <v>0.41</v>
@@ -3425,7 +3439,7 @@
       <c r="C9" s="1"/>
       <c r="I9" s="19">
         <f>Données!A7</f>
-        <v>180294</v>
+        <v>181917</v>
       </c>
       <c r="J9" s="20"/>
       <c r="K9" s="21">
@@ -3477,7 +3491,7 @@
       <c r="E14" s="109"/>
       <c r="F14" s="82">
         <f>IF((F4-E8-F10)&lt;0,0-F11,F4-E8-F12)</f>
-        <v>1551.1854750000002</v>
+        <v>1501.8150000000001</v>
       </c>
       <c r="I14" s="28" t="s">
         <v>92</v>
@@ -3502,7 +3516,7 @@
       </c>
       <c r="F16" s="45">
         <f>'Simulateur impôt simplifié 2025'!J35-('Simulateur impôt simplifié 2025'!F4*0.4525)</f>
-        <v>-52.195475000000101</v>
+        <v>-36.815000000000055</v>
       </c>
       <c r="I16" s="28"/>
     </row>
@@ -3512,7 +3526,7 @@
       </c>
       <c r="B17" s="14">
         <f>IF(B7/B6&lt;'Simulateur impôt simplifié 2025'!J5,0,IF(B7/B6&lt;'Simulateur impôt simplifié 2025'!J6,(B7/B6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6*'Simulateur impôt simplifié 2025'!B6,IF(B7/B6&lt;'Simulateur impôt simplifié 2025'!J7,((B7/B6-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B6,IF(B7/B6&lt;'Simulateur impôt simplifié 2025'!J8,((B7/B6-'Simulateur impôt simplifié 2025'!I8)*'Simulateur impôt simplifié 2025'!K8+('Simulateur impôt simplifié 2025'!J7-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B6,((B7/B6-'Simulateur impôt simplifié 2025'!I9)*'Simulateur impôt simplifié 2025'!K9+('Simulateur impôt simplifié 2025'!J8-'Simulateur impôt simplifié 2025'!I8)*'Simulateur impôt simplifié 2025'!K8+('Simulateur impôt simplifié 2025'!J7-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B6))))</f>
-        <v>2079.9900000000002</v>
+        <v>2046</v>
       </c>
       <c r="C17" s="13"/>
       <c r="E17" s="13" t="s">
@@ -3520,7 +3534,7 @@
       </c>
       <c r="F17" s="45">
         <f>'Simulateur impôt simplifié 2025'!J36-('Simulateur impôt simplifié 2025'!F4*0.4525)</f>
-        <v>528.8045249999999</v>
+        <v>544.18499999999995</v>
       </c>
       <c r="I17" s="29"/>
     </row>
@@ -3530,7 +3544,7 @@
       </c>
       <c r="B18" s="14">
         <f>IF(B7/B16&lt;'Simulateur impôt simplifié 2025'!J5,0,IF(B7/B16&lt;'Simulateur impôt simplifié 2025'!J6,(B7/B16-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6*'Simulateur impôt simplifié 2025'!B16,IF(B7/B16&lt;'Simulateur impôt simplifié 2025'!J7,((B7/B16-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B16,IF(B7/B16&lt;'Simulateur impôt simplifié 2025'!J8,((B7/B16-'Simulateur impôt simplifié 2025'!I8)*'Simulateur impôt simplifié 2025'!K8+('Simulateur impôt simplifié 2025'!J7-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B16,((B7/B16-'Simulateur impôt simplifié 2025'!I9)*'Simulateur impôt simplifié 2025'!K9+('Simulateur impôt simplifié 2025'!J8-'Simulateur impôt simplifié 2025'!I8)*'Simulateur impôt simplifié 2025'!K8+('Simulateur impôt simplifié 2025'!J7-'Simulateur impôt simplifié 2025'!I7)*'Simulateur impôt simplifié 2025'!K7+('Simulateur impôt simplifié 2025'!J6-'Simulateur impôt simplifié 2025'!I6)*'Simulateur impôt simplifié 2025'!K6)*'Simulateur impôt simplifié 2025'!B16))))-(B6-B16)*'Simulateur impôt simplifié 2025'!J22</f>
-        <v>-237.34000000000015</v>
+        <v>-292</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -3546,7 +3560,7 @@
       </c>
       <c r="J21" s="31">
         <f>Données!B17</f>
-        <v>1791</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3556,7 +3570,7 @@
       </c>
       <c r="J22" s="32">
         <f>Données!B18</f>
-        <v>3582</v>
+        <v>3614</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>

</xml_diff>